<commit_message>
feat(tactical): UI compaction, collapsible sidebar, pale map with schedule/KM, zone clustering & int64 pandas fix
- Fix pandas int64 TypeError when updating coordinates in solver and geocoding endpoints
- Collapse routes by default and show only active cargo/warehouses on load
- Add collapsible sidebar toggle [ - ] / [ + ] in DashboardLayout
- Map improvements: renamed to MAPA, pale desaturated base tiles, fixed selected badge contrast, route KM & return schedule stats
- Solver: Clarke & Wright SAVINGS + angular penalization for cluster strategy, distribution golden rule prioritizing distant customers
</commit_message>
<xml_diff>
--- a/Ficheiros EXCEL/TNB/GeoRoutePlan_TNB.xlsx
+++ b/Ficheiros EXCEL/TNB/GeoRoutePlan_TNB.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\01 - Paulo Batista\TESTE GeoRoutePlan\TNB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paulo\.gemini\antigravity\playground\core-omega\PRJT_GEO\Ficheiros EXCEL\TNB\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C910119-6667-4CE8-8EE6-C8E7D62183CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="825" yWindow="-16200" windowWidth="27165" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Armazéns" sheetId="1" r:id="rId1"/>

</xml_diff>